<commit_message>
Add stem number per plant to OBS data
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/GxExM/TillerAppearance.xlsx
+++ b/Tests/Validation/Wheat/GxExM/TillerAppearance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau-my.sharepoint.com/personal/hut104_csiro_au/Documents/Work/GRDC WheatYieldPhysiology/Simulations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Repos\ApsimX\Tests\Validation\Wheat\GxExM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_F25DC773A252ABDACC1048AAB99D5F285ADE58FC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F76569FD-5039-4863-8619-72E4EDCE908E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257388BC-35DF-42DC-9C6B-5D6FD6DA6072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Observed" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="53">
   <si>
     <t>SimulationName</t>
   </si>
@@ -192,6 +192,9 @@
   </si>
   <si>
     <t>Gatton2014CVSunstate</t>
+  </si>
+  <si>
+    <t>Wheat.Leaf.StemNumberPerPlant</t>
   </si>
 </sst>
 </file>
@@ -510,15 +513,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D212"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="27.265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -531,8 +534,11 @@
       <c r="D1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -543,7 +549,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -556,8 +562,12 @@
       <c r="D3">
         <v>1.0833333333333333</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E3">
+        <f>D3+1</f>
+        <v>2.083333333333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -570,8 +580,12 @@
       <c r="D4">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E4">
+        <f t="shared" ref="E4:E67" si="0">D4+1</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -584,8 +598,12 @@
       <c r="D5">
         <v>3.8333333333333335</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>4.8333333333333339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -598,8 +616,12 @@
       <c r="D6">
         <v>2.75</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -612,8 +634,12 @@
       <c r="D7">
         <v>3.1666666666666665</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666661</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -626,8 +652,12 @@
       <c r="D8">
         <v>3.125</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>4.125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -640,8 +670,12 @@
       <c r="D9">
         <v>3.6666666666666665</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>4.6666666666666661</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -652,7 +686,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -665,8 +699,12 @@
       <c r="D11">
         <v>1.1818181818181819</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>2.1818181818181817</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -679,8 +717,12 @@
       <c r="D12">
         <v>2.3636363636363638</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>3.3636363636363638</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -693,8 +735,12 @@
       <c r="D13">
         <v>4.666666666666667</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>5.666666666666667</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -707,8 +753,12 @@
       <c r="D14">
         <v>5.083333333333333</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>6.083333333333333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -721,8 +771,12 @@
       <c r="D15">
         <v>3.6666666666666665</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>4.6666666666666661</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -735,8 +789,12 @@
       <c r="D16">
         <v>4.416666666666667</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>5.416666666666667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -749,8 +807,12 @@
       <c r="D17">
         <v>3.5833333333333335</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>4.5833333333333339</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -763,8 +825,12 @@
       <c r="D18">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -775,7 +841,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -788,8 +854,12 @@
       <c r="D20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -802,8 +872,12 @@
       <c r="D21">
         <v>1.875</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>2.875</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -816,8 +890,12 @@
       <c r="D22">
         <v>3.3333333333333335</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>4.3333333333333339</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -830,8 +908,12 @@
       <c r="D23">
         <v>3</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -844,8 +926,12 @@
       <c r="D24">
         <v>3.3333333333333335</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E24">
+        <f t="shared" si="0"/>
+        <v>4.3333333333333339</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -858,8 +944,12 @@
       <c r="D25">
         <v>2.9166666666666665</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>3.9166666666666665</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -872,8 +962,12 @@
       <c r="D26">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -884,7 +978,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -897,8 +991,12 @@
       <c r="D28">
         <v>1.6363636363636365</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E28">
+        <f t="shared" si="0"/>
+        <v>2.6363636363636367</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -911,8 +1009,12 @@
       <c r="D29">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E29">
+        <f t="shared" si="0"/>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -925,8 +1027,12 @@
       <c r="D30">
         <v>4.583333333333333</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E30">
+        <f t="shared" si="0"/>
+        <v>5.583333333333333</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -939,8 +1045,12 @@
       <c r="D31">
         <v>5.583333333333333</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E31">
+        <f t="shared" si="0"/>
+        <v>6.583333333333333</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -953,8 +1063,12 @@
       <c r="D32">
         <v>5.5454545454545459</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>6.5454545454545459</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -967,8 +1081,12 @@
       <c r="D33">
         <v>4.166666666666667</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E33">
+        <f t="shared" si="0"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -981,8 +1099,12 @@
       <c r="D34">
         <v>4.166666666666667</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E34">
+        <f t="shared" si="0"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>5</v>
       </c>
@@ -993,7 +1115,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -1006,8 +1128,12 @@
       <c r="D36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E36">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>5</v>
       </c>
@@ -1020,8 +1146,12 @@
       <c r="D37">
         <v>1.9166666666666667</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E37">
+        <f t="shared" si="0"/>
+        <v>2.916666666666667</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -1034,8 +1164,12 @@
       <c r="D38">
         <v>3.9166666666666665</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E38">
+        <f t="shared" si="0"/>
+        <v>4.9166666666666661</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -1048,8 +1182,12 @@
       <c r="D39">
         <v>3.0833333333333335</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E39">
+        <f t="shared" si="0"/>
+        <v>4.0833333333333339</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -1062,8 +1200,12 @@
       <c r="D40">
         <v>5.416666666666667</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E40">
+        <f t="shared" si="0"/>
+        <v>6.416666666666667</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>5</v>
       </c>
@@ -1076,8 +1218,12 @@
       <c r="D41">
         <v>4</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E41">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>5</v>
       </c>
@@ -1090,8 +1236,12 @@
       <c r="D42">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E42">
+        <f t="shared" si="0"/>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>5</v>
       </c>
@@ -1104,8 +1254,12 @@
       <c r="D43">
         <v>3.5833333333333335</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E43">
+        <f t="shared" si="0"/>
+        <v>4.5833333333333339</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -1116,7 +1270,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -1129,8 +1283,12 @@
       <c r="D45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E45">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -1143,8 +1301,12 @@
       <c r="D46">
         <v>1.6666666666666667</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E46">
+        <f t="shared" si="0"/>
+        <v>2.666666666666667</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -1157,8 +1319,12 @@
       <c r="D47">
         <v>3.75</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E47">
+        <f t="shared" si="0"/>
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -1171,8 +1337,12 @@
       <c r="D48">
         <v>3.8333333333333335</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E48">
+        <f t="shared" si="0"/>
+        <v>4.8333333333333339</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1185,8 +1355,12 @@
       <c r="D49">
         <v>3.1666666666666665</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E49">
+        <f t="shared" si="0"/>
+        <v>4.1666666666666661</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -1199,8 +1373,12 @@
       <c r="D50">
         <v>3.4545454545454546</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E50">
+        <f t="shared" si="0"/>
+        <v>4.454545454545455</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>6</v>
       </c>
@@ -1213,8 +1391,12 @@
       <c r="D51">
         <v>2.9166666666666665</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E51">
+        <f t="shared" si="0"/>
+        <v>3.9166666666666665</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -1225,7 +1407,7 @@
         <v>42213</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>7</v>
       </c>
@@ -1236,7 +1418,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>7</v>
       </c>
@@ -1249,8 +1431,12 @@
       <c r="D54">
         <v>1.4</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E54">
+        <f t="shared" si="0"/>
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>7</v>
       </c>
@@ -1263,8 +1449,12 @@
       <c r="D55">
         <v>1.9166666666666667</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E55">
+        <f t="shared" si="0"/>
+        <v>2.916666666666667</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>7</v>
       </c>
@@ -1277,8 +1467,12 @@
       <c r="D56">
         <v>3.9166666666666665</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E56">
+        <f t="shared" si="0"/>
+        <v>4.9166666666666661</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>7</v>
       </c>
@@ -1291,8 +1485,12 @@
       <c r="D57">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E57">
+        <f t="shared" si="0"/>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -1305,8 +1503,12 @@
       <c r="D58">
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E58">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>7</v>
       </c>
@@ -1319,8 +1521,12 @@
       <c r="D59">
         <v>3</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E59">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -1333,8 +1539,12 @@
       <c r="D60">
         <v>2.75</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E60">
+        <f t="shared" si="0"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -1345,7 +1555,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -1358,8 +1568,12 @@
       <c r="D62">
         <v>1.1428571428571428</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E62">
+        <f t="shared" si="0"/>
+        <v>2.1428571428571428</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1372,8 +1586,12 @@
       <c r="D63">
         <v>2.4166666666666665</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E63">
+        <f t="shared" si="0"/>
+        <v>3.4166666666666665</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -1386,8 +1604,12 @@
       <c r="D64">
         <v>3.8</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E64">
+        <f t="shared" si="0"/>
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -1400,8 +1622,12 @@
       <c r="D65">
         <v>4.75</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E65">
+        <f t="shared" si="0"/>
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -1414,8 +1640,12 @@
       <c r="D66">
         <v>4</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E66">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>8</v>
       </c>
@@ -1428,8 +1658,12 @@
       <c r="D67">
         <v>4.166666666666667</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E67">
+        <f t="shared" si="0"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>8</v>
       </c>
@@ -1442,8 +1676,12 @@
       <c r="D68">
         <v>4.083333333333333</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E68">
+        <f t="shared" ref="E68:E131" si="1">D68+1</f>
+        <v>5.083333333333333</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>8</v>
       </c>
@@ -1456,8 +1694,12 @@
       <c r="D69">
         <v>4.25</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E69">
+        <f t="shared" si="1"/>
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>9</v>
       </c>
@@ -1468,7 +1710,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -1481,8 +1723,12 @@
       <c r="D71">
         <v>1.25</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E71">
+        <f t="shared" si="1"/>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -1495,8 +1741,12 @@
       <c r="D72">
         <v>2.0833333333333335</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E72">
+        <f t="shared" si="1"/>
+        <v>3.0833333333333335</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>9</v>
       </c>
@@ -1509,8 +1759,12 @@
       <c r="D73">
         <v>3</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E73">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>9</v>
       </c>
@@ -1523,8 +1777,12 @@
       <c r="D74">
         <v>4</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E74">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>9</v>
       </c>
@@ -1537,8 +1795,12 @@
       <c r="D75">
         <v>3.8333333333333335</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E75">
+        <f t="shared" si="1"/>
+        <v>4.8333333333333339</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>9</v>
       </c>
@@ -1551,8 +1813,12 @@
       <c r="D76">
         <v>3.3333333333333335</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E76">
+        <f t="shared" si="1"/>
+        <v>4.3333333333333339</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>9</v>
       </c>
@@ -1565,8 +1831,12 @@
       <c r="D77">
         <v>4.25</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E77">
+        <f t="shared" si="1"/>
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>9</v>
       </c>
@@ -1579,8 +1849,12 @@
       <c r="D78">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E78">
+        <f t="shared" si="1"/>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>10</v>
       </c>
@@ -1591,7 +1865,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>10</v>
       </c>
@@ -1604,8 +1878,12 @@
       <c r="D80">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E80">
+        <f t="shared" si="1"/>
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>10</v>
       </c>
@@ -1618,8 +1896,12 @@
       <c r="D81">
         <v>2.1666666666666665</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E81">
+        <f t="shared" si="1"/>
+        <v>3.1666666666666665</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>10</v>
       </c>
@@ -1632,8 +1914,12 @@
       <c r="D82">
         <v>3.6666666666666665</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E82">
+        <f t="shared" si="1"/>
+        <v>4.6666666666666661</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>10</v>
       </c>
@@ -1646,8 +1932,12 @@
       <c r="D83">
         <v>4.416666666666667</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E83">
+        <f t="shared" si="1"/>
+        <v>5.416666666666667</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>10</v>
       </c>
@@ -1660,8 +1950,12 @@
       <c r="D84">
         <v>2.75</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E84">
+        <f t="shared" si="1"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>10</v>
       </c>
@@ -1674,8 +1968,12 @@
       <c r="D85">
         <v>3</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E85">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>10</v>
       </c>
@@ -1688,8 +1986,12 @@
       <c r="D86">
         <v>3</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E86">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>11</v>
       </c>
@@ -1700,7 +2002,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>11</v>
       </c>
@@ -1713,8 +2015,12 @@
       <c r="D88">
         <v>1.0909090909090908</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E88">
+        <f t="shared" si="1"/>
+        <v>2.0909090909090908</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>11</v>
       </c>
@@ -1727,8 +2033,12 @@
       <c r="D89">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E89">
+        <f t="shared" si="1"/>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>11</v>
       </c>
@@ -1741,8 +2051,12 @@
       <c r="D90">
         <v>4.333333333333333</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E90">
+        <f t="shared" si="1"/>
+        <v>5.333333333333333</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>11</v>
       </c>
@@ -1755,8 +2069,12 @@
       <c r="D91">
         <v>4</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E91">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>11</v>
       </c>
@@ -1769,8 +2087,12 @@
       <c r="D92">
         <v>3.6666666666666665</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E92">
+        <f t="shared" si="1"/>
+        <v>4.6666666666666661</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>11</v>
       </c>
@@ -1783,8 +2105,12 @@
       <c r="D93">
         <v>3.1666666666666665</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E93">
+        <f t="shared" si="1"/>
+        <v>4.1666666666666661</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>11</v>
       </c>
@@ -1797,8 +2123,12 @@
       <c r="D94">
         <v>4</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E94">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>11</v>
       </c>
@@ -1811,8 +2141,12 @@
       <c r="D95">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E95">
+        <f t="shared" si="1"/>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>12</v>
       </c>
@@ -1823,7 +2157,7 @@
         <v>42160</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>12</v>
       </c>
@@ -1836,8 +2170,12 @@
       <c r="D97">
         <v>1</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E97">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>12</v>
       </c>
@@ -1850,8 +2188,12 @@
       <c r="D98">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E98">
+        <f t="shared" si="1"/>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>12</v>
       </c>
@@ -1864,8 +2206,12 @@
       <c r="D99">
         <v>3.4166666666666665</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E99">
+        <f t="shared" si="1"/>
+        <v>4.4166666666666661</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>12</v>
       </c>
@@ -1878,8 +2224,12 @@
       <c r="D100">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E100">
+        <f t="shared" si="1"/>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>12</v>
       </c>
@@ -1892,8 +2242,12 @@
       <c r="D101">
         <v>3.75</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E101">
+        <f t="shared" si="1"/>
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>12</v>
       </c>
@@ -1906,8 +2260,12 @@
       <c r="D102">
         <v>3</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E102">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>12</v>
       </c>
@@ -1920,8 +2278,12 @@
       <c r="D103">
         <v>3.9166666666666665</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E103">
+        <f t="shared" si="1"/>
+        <v>4.9166666666666661</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>28</v>
       </c>
@@ -1934,8 +2296,12 @@
       <c r="D104">
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E104">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>29</v>
       </c>
@@ -1948,8 +2314,12 @@
       <c r="D105">
         <v>0</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E105">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>30</v>
       </c>
@@ -1962,8 +2332,12 @@
       <c r="D106">
         <v>0</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E106">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>31</v>
       </c>
@@ -1976,8 +2350,12 @@
       <c r="D107">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E107">
+        <f t="shared" si="1"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>32</v>
       </c>
@@ -1990,8 +2368,12 @@
       <c r="D108">
         <v>0</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E108">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>33</v>
       </c>
@@ -2004,8 +2386,12 @@
       <c r="D109">
         <v>0</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E109">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>34</v>
       </c>
@@ -2018,8 +2404,12 @@
       <c r="D110">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E110">
+        <f t="shared" si="1"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>35</v>
       </c>
@@ -2032,8 +2422,12 @@
       <c r="D111">
         <v>0</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E111">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>36</v>
       </c>
@@ -2046,8 +2440,12 @@
       <c r="D112">
         <v>8.3333333333333329E-2</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E112">
+        <f t="shared" si="1"/>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>37</v>
       </c>
@@ -2060,8 +2458,12 @@
       <c r="D113">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E113">
+        <f t="shared" si="1"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>38</v>
       </c>
@@ -2074,8 +2476,12 @@
       <c r="D114">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E114">
+        <f t="shared" si="1"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>39</v>
       </c>
@@ -2088,8 +2494,12 @@
       <c r="D115">
         <v>8.3333333333333329E-2</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E115">
+        <f t="shared" si="1"/>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>28</v>
       </c>
@@ -2102,8 +2512,12 @@
       <c r="D116">
         <v>1.4166666666666667</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E116">
+        <f t="shared" si="1"/>
+        <v>2.416666666666667</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>29</v>
       </c>
@@ -2116,8 +2530,12 @@
       <c r="D117">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E117">
+        <f t="shared" si="1"/>
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>30</v>
       </c>
@@ -2130,8 +2548,12 @@
       <c r="D118">
         <v>1.0833333333333333</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E118">
+        <f t="shared" si="1"/>
+        <v>2.083333333333333</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>31</v>
       </c>
@@ -2144,8 +2566,12 @@
       <c r="D119">
         <v>1.3333333333333333</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E119">
+        <f t="shared" si="1"/>
+        <v>2.333333333333333</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>32</v>
       </c>
@@ -2158,8 +2584,12 @@
       <c r="D120">
         <v>1.25</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E120">
+        <f t="shared" si="1"/>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>33</v>
       </c>
@@ -2172,8 +2602,12 @@
       <c r="D121">
         <v>1.0833333333333333</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E121">
+        <f t="shared" si="1"/>
+        <v>2.083333333333333</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>34</v>
       </c>
@@ -2186,8 +2620,12 @@
       <c r="D122">
         <v>1.5833333333333333</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E122">
+        <f t="shared" si="1"/>
+        <v>2.583333333333333</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>35</v>
       </c>
@@ -2200,8 +2638,12 @@
       <c r="D123">
         <v>1.8333333333333333</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E123">
+        <f t="shared" si="1"/>
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>36</v>
       </c>
@@ -2214,8 +2656,12 @@
       <c r="D124">
         <v>1.75</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E124">
+        <f t="shared" si="1"/>
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>37</v>
       </c>
@@ -2228,8 +2674,12 @@
       <c r="D125">
         <v>1.75</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E125">
+        <f t="shared" si="1"/>
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>38</v>
       </c>
@@ -2242,8 +2692,12 @@
       <c r="D126">
         <v>1.4166666666666667</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E126">
+        <f t="shared" si="1"/>
+        <v>2.416666666666667</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>39</v>
       </c>
@@ -2256,8 +2710,12 @@
       <c r="D127">
         <v>1.8333333333333333</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E127">
+        <f t="shared" si="1"/>
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>28</v>
       </c>
@@ -2270,8 +2728,12 @@
       <c r="D128">
         <v>2.3333333333333335</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E128">
+        <f t="shared" si="1"/>
+        <v>3.3333333333333335</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>29</v>
       </c>
@@ -2284,8 +2746,12 @@
       <c r="D129">
         <v>2.1666666666666665</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E129">
+        <f t="shared" si="1"/>
+        <v>3.1666666666666665</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>30</v>
       </c>
@@ -2298,8 +2764,12 @@
       <c r="D130">
         <v>1.9166666666666667</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E130">
+        <f t="shared" si="1"/>
+        <v>2.916666666666667</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>31</v>
       </c>
@@ -2312,8 +2782,12 @@
       <c r="D131">
         <v>2.4166666666666665</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E131">
+        <f t="shared" si="1"/>
+        <v>3.4166666666666665</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -2326,8 +2800,12 @@
       <c r="D132">
         <v>2.0833333333333335</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E132">
+        <f t="shared" ref="E132:E195" si="2">D132+1</f>
+        <v>3.0833333333333335</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>33</v>
       </c>
@@ -2340,8 +2818,12 @@
       <c r="D133">
         <v>2.0833333333333335</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E133">
+        <f t="shared" si="2"/>
+        <v>3.0833333333333335</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>34</v>
       </c>
@@ -2354,8 +2836,12 @@
       <c r="D134">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E134">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>35</v>
       </c>
@@ -2368,8 +2854,12 @@
       <c r="D135">
         <v>2.9166666666666665</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E135">
+        <f t="shared" si="2"/>
+        <v>3.9166666666666665</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>36</v>
       </c>
@@ -2382,8 +2872,12 @@
       <c r="D136">
         <v>2.5833333333333335</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E136">
+        <f t="shared" si="2"/>
+        <v>3.5833333333333335</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>37</v>
       </c>
@@ -2396,8 +2890,12 @@
       <c r="D137">
         <v>2.5833333333333335</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E137">
+        <f t="shared" si="2"/>
+        <v>3.5833333333333335</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>38</v>
       </c>
@@ -2410,8 +2908,12 @@
       <c r="D138">
         <v>2.4166666666666665</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E138">
+        <f t="shared" si="2"/>
+        <v>3.4166666666666665</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>39</v>
       </c>
@@ -2424,8 +2926,12 @@
       <c r="D139">
         <v>2.6666666666666665</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E139">
+        <f t="shared" si="2"/>
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>28</v>
       </c>
@@ -2438,8 +2944,12 @@
       <c r="D140">
         <v>4.416666666666667</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E140">
+        <f t="shared" si="2"/>
+        <v>5.416666666666667</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>29</v>
       </c>
@@ -2452,8 +2962,12 @@
       <c r="D141">
         <v>4.25</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E141">
+        <f t="shared" si="2"/>
+        <v>5.25</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>30</v>
       </c>
@@ -2466,8 +2980,12 @@
       <c r="D142">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E142">
+        <f t="shared" si="2"/>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>31</v>
       </c>
@@ -2480,8 +2998,12 @@
       <c r="D143">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E143">
+        <f t="shared" si="2"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>32</v>
       </c>
@@ -2494,8 +3016,12 @@
       <c r="D144">
         <v>3.6666666666666665</v>
       </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E144">
+        <f t="shared" si="2"/>
+        <v>4.6666666666666661</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>33</v>
       </c>
@@ -2508,8 +3034,12 @@
       <c r="D145">
         <v>4.166666666666667</v>
       </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E145">
+        <f t="shared" si="2"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>34</v>
       </c>
@@ -2522,8 +3052,12 @@
       <c r="D146">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E146">
+        <f t="shared" si="2"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>35</v>
       </c>
@@ -2536,8 +3070,12 @@
       <c r="D147">
         <v>4.916666666666667</v>
       </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E147">
+        <f t="shared" si="2"/>
+        <v>5.916666666666667</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>36</v>
       </c>
@@ -2550,8 +3088,12 @@
       <c r="D148">
         <v>4.583333333333333</v>
       </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E148">
+        <f t="shared" si="2"/>
+        <v>5.583333333333333</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>37</v>
       </c>
@@ -2564,8 +3106,12 @@
       <c r="D149">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E149">
+        <f t="shared" si="2"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>38</v>
       </c>
@@ -2578,8 +3124,12 @@
       <c r="D150">
         <v>4.416666666666667</v>
       </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E150">
+        <f t="shared" si="2"/>
+        <v>5.416666666666667</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>39</v>
       </c>
@@ -2592,8 +3142,12 @@
       <c r="D151">
         <v>5.083333333333333</v>
       </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E151">
+        <f t="shared" si="2"/>
+        <v>6.083333333333333</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>34</v>
       </c>
@@ -2606,8 +3160,12 @@
       <c r="D152">
         <v>5</v>
       </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E152">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>40</v>
       </c>
@@ -2620,8 +3178,12 @@
       <c r="D153">
         <v>0</v>
       </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E153">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>41</v>
       </c>
@@ -2634,8 +3196,12 @@
       <c r="D154">
         <v>0</v>
       </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E154">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>42</v>
       </c>
@@ -2648,8 +3214,12 @@
       <c r="D155">
         <v>0</v>
       </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E155">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>43</v>
       </c>
@@ -2662,8 +3232,12 @@
       <c r="D156">
         <v>0</v>
       </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E156">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>44</v>
       </c>
@@ -2676,8 +3250,12 @@
       <c r="D157">
         <v>0</v>
       </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E157">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>45</v>
       </c>
@@ -2690,8 +3268,12 @@
       <c r="D158">
         <v>0</v>
       </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E158">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>46</v>
       </c>
@@ -2704,8 +3286,12 @@
       <c r="D159">
         <v>0</v>
       </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E159">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>47</v>
       </c>
@@ -2718,8 +3304,12 @@
       <c r="D160">
         <v>0</v>
       </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E160">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>48</v>
       </c>
@@ -2732,8 +3322,12 @@
       <c r="D161">
         <v>0</v>
       </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E161">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>49</v>
       </c>
@@ -2746,8 +3340,12 @@
       <c r="D162">
         <v>0</v>
       </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E162">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>50</v>
       </c>
@@ -2760,8 +3358,12 @@
       <c r="D163">
         <v>0</v>
       </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E163">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>51</v>
       </c>
@@ -2774,8 +3376,12 @@
       <c r="D164">
         <v>0</v>
       </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E164">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>40</v>
       </c>
@@ -2788,8 +3394,12 @@
       <c r="D165">
         <v>8.3333333333333329E-2</v>
       </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E165">
+        <f t="shared" si="2"/>
+        <v>1.0833333333333333</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>41</v>
       </c>
@@ -2802,8 +3412,12 @@
       <c r="D166">
         <v>0</v>
       </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E166">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>42</v>
       </c>
@@ -2816,8 +3430,12 @@
       <c r="D167">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E167">
+        <f t="shared" si="2"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>43</v>
       </c>
@@ -2830,8 +3448,12 @@
       <c r="D168">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E168">
+        <f t="shared" si="2"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>44</v>
       </c>
@@ -2844,8 +3466,12 @@
       <c r="D169">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E169">
+        <f t="shared" si="2"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>45</v>
       </c>
@@ -2858,8 +3484,12 @@
       <c r="D170">
         <v>0</v>
       </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E170">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>46</v>
       </c>
@@ -2872,8 +3502,12 @@
       <c r="D171">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E171">
+        <f t="shared" si="2"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>47</v>
       </c>
@@ -2886,8 +3520,12 @@
       <c r="D172">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E172">
+        <f t="shared" si="2"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>48</v>
       </c>
@@ -2900,8 +3538,12 @@
       <c r="D173">
         <v>0.33333333333333331</v>
       </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E173">
+        <f t="shared" si="2"/>
+        <v>1.3333333333333333</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>49</v>
       </c>
@@ -2914,8 +3556,12 @@
       <c r="D174">
         <v>0.58333333333333337</v>
       </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E174">
+        <f t="shared" si="2"/>
+        <v>1.5833333333333335</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>50</v>
       </c>
@@ -2928,8 +3574,12 @@
       <c r="D175">
         <v>0</v>
       </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E175">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>51</v>
       </c>
@@ -2942,8 +3592,12 @@
       <c r="D176">
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E176">
+        <f t="shared" si="2"/>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>40</v>
       </c>
@@ -2956,8 +3610,12 @@
       <c r="D177">
         <v>1.3333333333333333</v>
       </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E177">
+        <f t="shared" si="2"/>
+        <v>2.333333333333333</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>41</v>
       </c>
@@ -2970,8 +3628,12 @@
       <c r="D178">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E178">
+        <f t="shared" si="2"/>
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>42</v>
       </c>
@@ -2984,8 +3646,12 @@
       <c r="D179">
         <v>1.5833333333333333</v>
       </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E179">
+        <f t="shared" si="2"/>
+        <v>2.583333333333333</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>43</v>
       </c>
@@ -2998,8 +3664,12 @@
       <c r="D180">
         <v>1.75</v>
       </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E180">
+        <f t="shared" si="2"/>
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>44</v>
       </c>
@@ -3012,8 +3682,12 @@
       <c r="D181">
         <v>1.6666666666666667</v>
       </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E181">
+        <f t="shared" si="2"/>
+        <v>2.666666666666667</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>45</v>
       </c>
@@ -3026,8 +3700,12 @@
       <c r="D182">
         <v>1.3333333333333333</v>
       </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E182">
+        <f t="shared" si="2"/>
+        <v>2.333333333333333</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>46</v>
       </c>
@@ -3040,8 +3718,12 @@
       <c r="D183">
         <v>1.8333333333333333</v>
       </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E183">
+        <f t="shared" si="2"/>
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>47</v>
       </c>
@@ -3054,8 +3736,12 @@
       <c r="D184">
         <v>1.9166666666666667</v>
       </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E184">
+        <f t="shared" si="2"/>
+        <v>2.916666666666667</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>48</v>
       </c>
@@ -3068,8 +3754,12 @@
       <c r="D185">
         <v>2</v>
       </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E185">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>49</v>
       </c>
@@ -3082,8 +3772,12 @@
       <c r="D186">
         <v>1.8333333333333333</v>
       </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E186">
+        <f t="shared" si="2"/>
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>50</v>
       </c>
@@ -3096,8 +3790,12 @@
       <c r="D187">
         <v>1.9166666666666667</v>
       </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E187">
+        <f t="shared" si="2"/>
+        <v>2.916666666666667</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>51</v>
       </c>
@@ -3110,8 +3808,12 @@
       <c r="D188">
         <v>1.8333333333333333</v>
       </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E188">
+        <f t="shared" si="2"/>
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>40</v>
       </c>
@@ -3124,8 +3826,12 @@
       <c r="D189">
         <v>2.4166666666666665</v>
       </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E189">
+        <f t="shared" si="2"/>
+        <v>3.4166666666666665</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>41</v>
       </c>
@@ -3138,8 +3844,12 @@
       <c r="D190">
         <v>2.1666666666666665</v>
       </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E190">
+        <f t="shared" si="2"/>
+        <v>3.1666666666666665</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>42</v>
       </c>
@@ -3152,8 +3862,12 @@
       <c r="D191">
         <v>2.3333333333333335</v>
       </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E191">
+        <f t="shared" si="2"/>
+        <v>3.3333333333333335</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>43</v>
       </c>
@@ -3166,8 +3880,12 @@
       <c r="D192">
         <v>3</v>
       </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E192">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>44</v>
       </c>
@@ -3180,8 +3898,12 @@
       <c r="D193">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E193">
+        <f t="shared" si="2"/>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>45</v>
       </c>
@@ -3194,8 +3916,12 @@
       <c r="D194">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E194">
+        <f t="shared" si="2"/>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>46</v>
       </c>
@@ -3208,8 +3934,12 @@
       <c r="D195">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E195">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>47</v>
       </c>
@@ -3222,8 +3952,12 @@
       <c r="D196">
         <v>2.6666666666666665</v>
       </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E196">
+        <f t="shared" ref="E196:E212" si="3">D196+1</f>
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>48</v>
       </c>
@@ -3236,8 +3970,12 @@
       <c r="D197">
         <v>2.75</v>
       </c>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E197">
+        <f t="shared" si="3"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>49</v>
       </c>
@@ -3250,8 +3988,12 @@
       <c r="D198">
         <v>3.0833333333333335</v>
       </c>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E198">
+        <f t="shared" si="3"/>
+        <v>4.0833333333333339</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>50</v>
       </c>
@@ -3264,8 +4006,12 @@
       <c r="D199">
         <v>2.75</v>
       </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E199">
+        <f t="shared" si="3"/>
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>51</v>
       </c>
@@ -3278,8 +4024,12 @@
       <c r="D200">
         <v>2.5833333333333335</v>
       </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E200">
+        <f t="shared" si="3"/>
+        <v>3.5833333333333335</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>40</v>
       </c>
@@ -3292,8 +4042,12 @@
       <c r="D201">
         <v>3.25</v>
       </c>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E201">
+        <f t="shared" si="3"/>
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>41</v>
       </c>
@@ -3306,8 +4060,12 @@
       <c r="D202">
         <v>4.666666666666667</v>
       </c>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E202">
+        <f t="shared" si="3"/>
+        <v>5.666666666666667</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>42</v>
       </c>
@@ -3320,8 +4078,12 @@
       <c r="D203">
         <v>4.583333333333333</v>
       </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E203">
+        <f t="shared" si="3"/>
+        <v>5.583333333333333</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>43</v>
       </c>
@@ -3334,8 +4096,12 @@
       <c r="D204">
         <v>5</v>
       </c>
-    </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E204">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>44</v>
       </c>
@@ -3348,8 +4114,12 @@
       <c r="D205">
         <v>3.4166666666666665</v>
       </c>
-    </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E205">
+        <f t="shared" si="3"/>
+        <v>4.4166666666666661</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>45</v>
       </c>
@@ -3362,8 +4132,12 @@
       <c r="D206">
         <v>4.75</v>
       </c>
-    </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E206">
+        <f t="shared" si="3"/>
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>46</v>
       </c>
@@ -3376,8 +4150,12 @@
       <c r="D207">
         <v>4.166666666666667</v>
       </c>
-    </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E207">
+        <f t="shared" si="3"/>
+        <v>5.166666666666667</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>47</v>
       </c>
@@ -3390,8 +4168,12 @@
       <c r="D208">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E208">
+        <f t="shared" si="3"/>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>48</v>
       </c>
@@ -3404,8 +4186,12 @@
       <c r="D209">
         <v>4.416666666666667</v>
       </c>
-    </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E209">
+        <f t="shared" si="3"/>
+        <v>5.416666666666667</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>49</v>
       </c>
@@ -3418,8 +4204,12 @@
       <c r="D210">
         <v>4.583333333333333</v>
       </c>
-    </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E210">
+        <f t="shared" si="3"/>
+        <v>5.583333333333333</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>50</v>
       </c>
@@ -3432,8 +4222,12 @@
       <c r="D211">
         <v>4.833333333333333</v>
       </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E211">
+        <f t="shared" si="3"/>
+        <v>5.833333333333333</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>51</v>
       </c>
@@ -3446,8 +4240,16 @@
       <c r="D212">
         <v>4.5</v>
       </c>
+      <c r="E212">
+        <f t="shared" si="3"/>
+        <v>5.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 UNOFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 UNOFFICIAL</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>